<commit_message>
Baza korigirana, redizajn gumba Mim (nije zavrsen), Izmjena Genre party igre u vlakić
</commit_message>
<xml_diff>
--- a/bandhelper_final_ui_ready_v7_empty.xlsx
+++ b/bandhelper_final_ui_ready_v7_empty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markomarjanovic/Apps/Repertoar_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7108D085-39E9-6C47-BA4F-FC3CCBB8049B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDE3897-0D6A-774F-8084-C584E0114105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -113,9 +113,6 @@
     <t>Strano</t>
   </si>
   <si>
-    <t>Party igre</t>
-  </si>
-  <si>
     <t>Trash</t>
   </si>
   <si>
@@ -150,6 +147,9 @@
   </si>
   <si>
     <t>Proba</t>
+  </si>
+  <si>
+    <t>Vlakić</t>
   </si>
 </sst>
 </file>
@@ -959,7 +959,7 @@
         <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -973,13 +973,13 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -990,7 +990,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
         <v>26</v>
@@ -998,10 +998,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1009,15 +1009,15 @@
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -1025,7 +1025,7 @@
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1035,17 +1035,17 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>